<commit_message>
自动更新Excel文件 - Mon Sep 14 00:53:03 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>20260905</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,10 +1017,10 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1048,10 +1048,10 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1110,10 +1110,10 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20260908</v>
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1552,10 +1552,10 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1645,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1676,10 +1676,10 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,10 +1773,10 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,10 +1932,10 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F47" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20260908</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
         <v>20260909</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>20260909</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F52" t="n">
         <v>20260909</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
         <v>20260909</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
         <v>20260909</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
         <v>20260909</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
         <v>20260909</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
         <v>20260909</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20260908</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F65" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -2552,10 +2552,10 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
@@ -2583,10 +2583,10 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F68" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2614,10 +2614,10 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F69" t="n">
-        <v>20260904</v>
+        <v>20260914</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>20260905</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>20260905</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
         <v>20260905</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
         <v>20260905</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
         <v>20260905</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>20260905</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>20260905</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>20260908</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
         <v>20260908</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
         <v>20260908</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
         <v>20260908</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>20260908</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F82" t="n">
         <v>20260908</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F83" t="n">
         <v>20260908</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F84" t="n">
         <v>20260908</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>20260908</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>20260908</v>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20260907</v>
+        <v>20260914</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>20260908</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20260910</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
         <v>20260907</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
         <v>20260905</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>20260905</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>20260905</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" t="n">
         <v>20260905</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Sep 15 01:20:03 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20260908</v>
+        <v>20260915</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20260908</v>
+        <v>20260915</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
         <v>20260909</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>20260909</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>20260909</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>20260909</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>20260909</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>20260909</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>20260909</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
         <v>20260909</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20260908</v>
+        <v>20260915</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,10 +2645,10 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F70" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F71" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2738,10 +2738,10 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2769,10 +2769,10 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F76" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F77" t="n">
         <v>20260908</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F78" t="n">
         <v>20260908</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>20260908</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
         <v>20260908</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>20260908</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>20260908</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
         <v>20260908</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>20260908</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F85" t="n">
         <v>20260908</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F86" t="n">
         <v>20260908</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" t="n">
         <v>20260908</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20260910</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>20260907</v>
@@ -3451,10 +3451,10 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F96" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -3482,10 +3482,10 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F97" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F98" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3544,10 +3544,10 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F99" t="n">
-        <v>20260905</v>
+        <v>20260915</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Sep 16 01:15:29 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>20260909</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>20260909</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>20260909</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>20260909</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
         <v>20260909</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
         <v>20260909</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F56" t="n">
         <v>20260909</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>20260909</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77" t="n">
         <v>20260908</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
         <v>20260908</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>20260908</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
         <v>20260908</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
         <v>20260908</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82" t="n">
         <v>20260908</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F83" t="n">
         <v>20260908</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F84" t="n">
         <v>20260908</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F85" t="n">
         <v>20260908</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F86" t="n">
         <v>20260908</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F93" t="n">
         <v>20260908</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20260910</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" t="n">
         <v>20260907</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Sep 17 01:15:20 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F50" t="n">
         <v>20260909</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
         <v>20260909</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>20260909</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>20260909</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>20260909</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F55" t="n">
         <v>20260909</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>20260909</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
         <v>20260909</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F77" t="n">
         <v>20260908</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
         <v>20260908</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" t="n">
         <v>20260908</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" t="n">
         <v>20260908</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" t="n">
         <v>20260908</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" t="n">
         <v>20260908</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>20260908</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="n">
         <v>20260908</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" t="n">
         <v>20260908</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="n">
         <v>20260908</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" t="n">
         <v>20260908</v>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20260910</v>
+        <v>20260917</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,10 +3420,10 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F95" t="n">
-        <v>20260907</v>
+        <v>20260917</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Sep 18 01:10:52 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>20260909</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>20260909</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
         <v>20260909</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>20260909</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>20260909</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
         <v>20260909</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>20260909</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>20260909</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,10 +2862,10 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F77" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2893,10 +2893,10 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F78" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F79" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F81" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -3017,10 +3017,10 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F82" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -3048,10 +3048,10 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F83" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -3079,10 +3079,10 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F85" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -3141,10 +3141,10 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F86" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,10 +3358,10 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F93" t="n">
-        <v>20260908</v>
+        <v>20260918</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Sep 19 01:05:20 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,10 +2025,10 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F50" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2056,10 +2056,10 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F51" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2087,10 +2087,10 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2118,10 +2118,10 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F53" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2149,10 +2149,10 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F54" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2180,10 +2180,10 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F55" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2211,10 +2211,10 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F56" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -2242,10 +2242,10 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F57" t="n">
-        <v>20260909</v>
+        <v>20260919</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Sep 20 00:55:27 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>20260907</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>20260907</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>20260907</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>20260911</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>20260907</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>20260911</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>20260907</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>20260911</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20260914</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>20260907</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>20260911</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>20260907</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
         <v>20260907</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>20260907</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>20260911</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>20260911</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>20260911</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>20260911</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>20260911</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>20260911</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20260914</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20260914</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
         <v>20260911</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20260914</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>20260911</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20260914</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20260914</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20260914</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20260914</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20260914</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20260914</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>20260911</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20260914</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Mon Sep 21 00:57:59 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,10 +493,10 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -528,10 +528,10 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F3" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -563,10 +563,10 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -598,10 +598,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -633,10 +633,10 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -664,10 +664,10 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -695,10 +695,10 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -726,10 +726,10 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,10 +788,10 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -819,10 +819,10 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
@@ -850,10 +850,10 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -885,10 +885,10 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -920,10 +920,10 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>20260907</v>
+        <v>20260921</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,10 +986,10 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,10 +1141,10 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1172,10 +1172,10 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1234,10 +1234,10 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F25" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20260915</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,10 +1804,10 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F43" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,10 +1866,10 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F45" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20260915</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20260915</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,10 +3296,10 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F91" t="n">
-        <v>20260911</v>
+        <v>20260921</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20260914</v>
+        <v>20260921</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Sep 22 01:32:48 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20260915</v>
+        <v>20260922</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20260915</v>
+        <v>20260922</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>20260913</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>20260913</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
         <v>20260913</v>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20260915</v>
+        <v>20260922</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
         <v>20260913</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
         <v>20260913</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>20260913</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Sep 23 01:22:45 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>20260914</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>20260914</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>20260914</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>20260914</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>20260914</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>20260914</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>20260914</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>20260914</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>20260914</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>20260914</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>20260914</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
         <v>20260914</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>20260914</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
         <v>20260914</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>20260914</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
         <v>20260914</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>20260914</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,10 +2273,10 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F58" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -2304,10 +2304,10 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2335,10 +2335,10 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,10 +2397,10 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2428,10 +2428,10 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2459,10 +2459,10 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F64" t="n">
-        <v>20260913</v>
+        <v>20260923</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" t="n">
         <v>20260914</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" t="n">
         <v>20260914</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>20260914</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
         <v>20260914</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>20260914</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20260917</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Sep 24 01:16:52 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>20260915</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,10 +1017,10 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1048,10 +1048,10 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1110,10 +1110,10 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1552,10 +1552,10 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1645,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1676,10 +1676,10 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,10 +1773,10 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,10 +1932,10 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F47" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F65" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -2552,10 +2552,10 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
@@ -2583,10 +2583,10 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F68" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2614,10 +2614,10 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F69" t="n">
-        <v>20260914</v>
+        <v>20260924</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>20260915</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>20260915</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
         <v>20260915</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
         <v>20260915</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
         <v>20260915</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>20260915</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>20260915</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20260917</v>
+        <v>20260924</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
         <v>20260915</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>20260915</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>20260915</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" t="n">
         <v>20260915</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Sep 25 01:21:07 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,10 +2645,10 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F70" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F71" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2738,10 +2738,10 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2769,10 +2769,10 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F76" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,10 +3451,10 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F96" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -3482,10 +3482,10 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F97" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F98" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3544,10 +3544,10 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F99" t="n">
-        <v>20260915</v>
+        <v>20260925</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Sep 26 01:23:51 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" t="n">
         <v>20260917</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Sep 27 01:16:51 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20260921</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20260921</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20260921</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20260921</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20260921</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20260921</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F77" t="n">
         <v>20260918</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
         <v>20260918</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" t="n">
         <v>20260918</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" t="n">
         <v>20260918</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" t="n">
         <v>20260918</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" t="n">
         <v>20260918</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>20260918</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="n">
         <v>20260918</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" t="n">
         <v>20260918</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="n">
         <v>20260918</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20260921</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20260921</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20260921</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20260921</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20260921</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" t="n">
         <v>20260918</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,10 +3420,10 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F95" t="n">
-        <v>20260917</v>
+        <v>20260927</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Mon Sep 28 01:30:40 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20260922</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20260922</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>20260919</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>20260919</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
         <v>20260919</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>20260919</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>20260919</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
         <v>20260919</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>20260919</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>20260919</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20260922</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,10 +2862,10 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F77" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2893,10 +2893,10 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F78" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F79" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F81" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -3017,10 +3017,10 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F82" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -3048,10 +3048,10 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F83" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -3079,10 +3079,10 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F85" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -3141,10 +3141,10 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F86" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20260921</v>
+        <v>20260928</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,10 +3358,10 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F93" t="n">
-        <v>20260918</v>
+        <v>20260928</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Sep 29 02:32:41 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20260922</v>
+        <v>20260929</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20260922</v>
+        <v>20260929</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,10 +2025,10 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F50" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2056,10 +2056,10 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F51" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2087,10 +2087,10 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2118,10 +2118,10 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F53" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2149,10 +2149,10 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F54" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2180,10 +2180,10 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F55" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2211,10 +2211,10 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F56" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -2242,10 +2242,10 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F57" t="n">
-        <v>20260919</v>
+        <v>20260929</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20260922</v>
+        <v>20260929</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Sep 30 01:57:20 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>20260921</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>20260921</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>20260921</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>20260921</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>20260921</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>20260921</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>20260921</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>20260921</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>20260921</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>20260921</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
         <v>20260921</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>20260921</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>20260921</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20260924</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Oct  1 01:57:48 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,10 +598,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,10 +664,10 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,10 +726,10 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,10 +819,10 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,10 +986,10 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,10 +1141,10 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1172,10 +1172,10 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1234,10 +1234,10 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F25" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,10 +1804,10 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F43" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,10 +1866,10 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F45" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,10 +3296,10 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F91" t="n">
-        <v>20260921</v>
+        <v>20261001</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20260924</v>
+        <v>20261001</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Oct  2 02:06:09 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>20260923</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>20260923</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
         <v>20260923</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
         <v>20260923</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
         <v>20260923</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>20260923</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Oct  3 01:51:06 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>20260924</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>20260924</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>20260924</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>20260924</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>20260924</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>20260924</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>20260924</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>20260924</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>20260924</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>20260924</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>20260924</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
         <v>20260924</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>20260924</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
         <v>20260924</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>20260924</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
         <v>20260924</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>20260924</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,10 +2273,10 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F58" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -2304,10 +2304,10 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2335,10 +2335,10 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,10 +2397,10 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2428,10 +2428,10 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2459,10 +2459,10 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F64" t="n">
-        <v>20260923</v>
+        <v>20261003</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" t="n">
         <v>20260924</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" t="n">
         <v>20260924</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>20260924</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
         <v>20260924</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>20260924</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Oct  4 02:29:51 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>20260921</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>20260921</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>20260921</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>20260921</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>20260921</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20260928</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>20260921</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>20260921</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
         <v>20260921</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>20260921</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>20260925</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,10 +1017,10 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1048,10 +1048,10 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1110,10 +1110,10 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1552,10 +1552,10 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1645,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1676,10 +1676,10 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20260928</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20260928</v>
@@ -1773,10 +1773,10 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20260928</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20260928</v>
@@ -1932,10 +1932,10 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F47" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20260928</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F65" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -2552,10 +2552,10 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
@@ -2583,10 +2583,10 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F68" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2614,10 +2614,10 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F69" t="n">
-        <v>20260924</v>
+        <v>20261004</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>20260925</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>20260925</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
         <v>20260925</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
         <v>20260925</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
         <v>20260925</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>20260925</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>20260925</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20260928</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20260928</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20260928</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20260928</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20260928</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
         <v>20260925</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>20260925</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>20260925</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" t="n">
         <v>20260925</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Mon Oct  5 01:46:55 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,10 +493,10 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -528,10 +528,10 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F3" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -563,10 +563,10 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,10 +633,10 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,10 +695,10 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,10 +788,10 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,10 +850,10 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -885,10 +885,10 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -920,10 +920,10 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>20260921</v>
+        <v>20261005</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20260929</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20260929</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20260929</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,10 +2645,10 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F70" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F71" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2738,10 +2738,10 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2769,10 +2769,10 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F76" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20260928</v>
+        <v>20261005</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,10 +3451,10 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F96" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -3482,10 +3482,10 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F97" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F98" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3544,10 +3544,10 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F99" t="n">
-        <v>20260925</v>
+        <v>20261005</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Oct  6 02:50:38 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20260929</v>
+        <v>20261006</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20260929</v>
+        <v>20261006</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20260929</v>
+        <v>20261006</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" t="n">
         <v>20260927</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Oct  7 02:12:24 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F77" t="n">
         <v>20260928</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
         <v>20260928</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" t="n">
         <v>20260928</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" t="n">
         <v>20260928</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" t="n">
         <v>20260928</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" t="n">
         <v>20260928</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>20260928</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="n">
         <v>20260928</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" t="n">
         <v>20260928</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="n">
         <v>20260928</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" t="n">
         <v>20260928</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20261001</v>
@@ -3420,10 +3420,10 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F95" t="n">
-        <v>20260927</v>
+        <v>20261007</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Oct  8 02:37:45 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>20260929</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>20260929</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
         <v>20260929</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>20260929</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>20260929</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
         <v>20260929</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>20260929</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>20260929</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,10 +2862,10 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F77" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2893,10 +2893,10 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F78" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F79" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F81" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -3017,10 +3017,10 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F82" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -3048,10 +3048,10 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F83" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -3079,10 +3079,10 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F85" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -3141,10 +3141,10 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F86" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,10 +3358,10 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F93" t="n">
-        <v>20260928</v>
+        <v>20261008</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20261001</v>
+        <v>20261008</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Oct  9 02:52:53 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,10 +2025,10 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F50" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2056,10 +2056,10 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F51" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2087,10 +2087,10 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2118,10 +2118,10 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F53" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2149,10 +2149,10 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F54" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2180,10 +2180,10 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F55" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2211,10 +2211,10 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F56" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -2242,10 +2242,10 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F57" t="n">
-        <v>20260929</v>
+        <v>20261009</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Oct 10 02:13:41 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>20261001</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>20261001</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>20261001</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>20261001</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>20261001</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>20261001</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>20261001</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>20261001</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>20261001</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>20261001</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
         <v>20261001</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>20261001</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>20261001</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Oct 11 01:45:51 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,10 +598,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,10 +664,10 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,10 +726,10 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20261005</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,10 +819,10 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,10 +986,10 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,10 +1141,10 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1172,10 +1172,10 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1234,10 +1234,10 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F25" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20261005</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20261005</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,10 +1804,10 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F43" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20261005</v>
@@ -1866,10 +1866,10 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F45" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20261005</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20261005</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20261005</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20261005</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20261005</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20261005</v>
@@ -3296,10 +3296,10 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F91" t="n">
-        <v>20261001</v>
+        <v>20261011</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20261005</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Mon Oct 12 02:13:16 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20261006</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20261006</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>20261003</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>20261003</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
         <v>20261003</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20261006</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
         <v>20261003</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
         <v>20261003</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>20261003</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20261005</v>
+        <v>20261012</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Oct 13 03:27:39 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>20261004</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>20261004</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>20261004</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>20261004</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20261006</v>
+        <v>20261013</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>20261004</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>20261004</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>20261004</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>20261004</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>20261004</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>20261004</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>20261004</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
         <v>20261004</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>20261004</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
         <v>20261004</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>20261004</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
         <v>20261004</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>20261004</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20261006</v>
+        <v>20261013</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,10 +2273,10 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F58" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -2304,10 +2304,10 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2335,10 +2335,10 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20261006</v>
+        <v>20261013</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,10 +2397,10 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2428,10 +2428,10 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2459,10 +2459,10 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F64" t="n">
-        <v>20261003</v>
+        <v>20261013</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" t="n">
         <v>20261004</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" t="n">
         <v>20261004</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>20261004</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
         <v>20261004</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>20261004</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Oct 14 01:45:25 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>20261005</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,10 +1017,10 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1048,10 +1048,10 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1110,10 +1110,10 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1552,10 +1552,10 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1645,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1676,10 +1676,10 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,10 +1773,10 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,10 +1932,10 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F47" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F65" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -2552,10 +2552,10 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
@@ -2583,10 +2583,10 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F68" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2614,10 +2614,10 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F69" t="n">
-        <v>20261004</v>
+        <v>20261014</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>20261005</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>20261005</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
         <v>20261005</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
         <v>20261005</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
         <v>20261005</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>20261005</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>20261005</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20261008</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
         <v>20261005</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>20261005</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>20261005</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" t="n">
         <v>20261005</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Oct 15 01:21:22 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,10 +2645,10 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F70" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F71" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2738,10 +2738,10 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2769,10 +2769,10 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F76" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20261008</v>
+        <v>20261015</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,10 +3451,10 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F96" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -3482,10 +3482,10 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F97" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F98" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3544,10 +3544,10 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F99" t="n">
-        <v>20261005</v>
+        <v>20261015</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Oct 16 01:07:33 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F95" t="n">
         <v>20261007</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Oct 17 01:12:57 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F77" t="n">
         <v>20261008</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F78" t="n">
         <v>20261008</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" t="n">
         <v>20261008</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F80" t="n">
         <v>20261008</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F81" t="n">
         <v>20261008</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" t="n">
         <v>20261008</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="n">
         <v>20261008</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F84" t="n">
         <v>20261008</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F85" t="n">
         <v>20261008</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="n">
         <v>20261008</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F93" t="n">
         <v>20261008</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,10 +3420,10 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F95" t="n">
-        <v>20261007</v>
+        <v>20261017</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Oct 18 00:48:08 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
         <v>20261005</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
         <v>20261005</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
         <v>20261005</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
         <v>20261005</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
         <v>20261005</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20261012</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
         <v>20261005</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="n">
         <v>20261005</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
         <v>20261005</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" t="n">
         <v>20261005</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20261012</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20261012</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20261012</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20261012</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20261012</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" t="n">
         <v>20261009</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F51" t="n">
         <v>20261009</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
         <v>20261009</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F53" t="n">
         <v>20261009</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="n">
         <v>20261009</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F55" t="n">
         <v>20261009</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F56" t="n">
         <v>20261009</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F57" t="n">
         <v>20261009</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,10 +2862,10 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F77" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -2893,10 +2893,10 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F78" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -2924,10 +2924,10 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F79" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -2955,10 +2955,10 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F80" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -2986,10 +2986,10 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F81" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr">
@@ -3017,10 +3017,10 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F82" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr">
@@ -3048,10 +3048,10 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F83" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr">
@@ -3079,10 +3079,10 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3110,10 +3110,10 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F85" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G85" t="inlineStr"/>
       <c r="H85" t="inlineStr">
@@ -3141,10 +3141,10 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F86" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20261012</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20261012</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20261012</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20261012</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20261012</v>
@@ -3358,10 +3358,10 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F93" t="n">
-        <v>20261008</v>
+        <v>20261018</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Mon Oct 19 01:00:39 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,10 +493,10 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F2" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -528,10 +528,10 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F3" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -563,10 +563,10 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F4" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,10 +633,10 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,10 +695,10 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,10 +757,10 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
@@ -788,10 +788,10 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F11" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,10 +850,10 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F13" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -885,10 +885,10 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F14" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -920,10 +920,10 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="F15" t="n">
-        <v>20261005</v>
+        <v>20261019</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="n">
         <v>20261013</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,10 +1711,10 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F40" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
@@ -1742,10 +1742,10 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F41" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,10 +1835,10 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F44" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,10 +1897,10 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,10 +1963,10 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F48" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F49" t="n">
         <v>20261013</v>
@@ -2025,10 +2025,10 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F50" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2056,10 +2056,10 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F51" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2087,10 +2087,10 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F52" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2118,10 +2118,10 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F53" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2149,10 +2149,10 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F54" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2180,10 +2180,10 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F55" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2211,10 +2211,10 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F56" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr">
@@ -2242,10 +2242,10 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F57" t="n">
-        <v>20261009</v>
+        <v>20261019</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F61" t="n">
         <v>20261013</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,10 +3172,10 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F87" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -3203,10 +3203,10 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F88" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G88" t="inlineStr"/>
       <c r="H88" t="inlineStr">
@@ -3234,10 +3234,10 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F89" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G89" t="inlineStr"/>
       <c r="H89" t="inlineStr">
@@ -3265,10 +3265,10 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F90" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G90" t="inlineStr"/>
       <c r="H90" t="inlineStr">
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,10 +3327,10 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F92" t="n">
-        <v>20261012</v>
+        <v>20261019</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Tue Oct 20 01:40:20 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
         <v>20261011</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="n">
         <v>20261011</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" t="n">
         <v>20261011</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
         <v>20261011</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" t="n">
         <v>20261011</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F22" t="n">
         <v>20261011</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
         <v>20261011</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F24" t="n">
         <v>20261011</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F25" t="n">
         <v>20261011</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F26" t="n">
         <v>20261011</v>
@@ -1296,10 +1296,10 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F27" t="n">
-        <v>20261013</v>
+        <v>20261020</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="n">
         <v>20261011</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
         <v>20261011</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,10 +1994,10 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F49" t="n">
-        <v>20261013</v>
+        <v>20261020</v>
       </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,10 +2366,10 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F61" t="n">
-        <v>20261013</v>
+        <v>20261020</v>
       </c>
       <c r="G61" t="inlineStr"/>
       <c r="H61" t="inlineStr">
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F91" t="n">
         <v>20261011</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Wed Oct 21 01:25:44 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,10 +598,10 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,10 +664,10 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F7" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,10 +726,10 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,10 +819,10 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,10 +986,10 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F17" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,10 +1141,10 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F22" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1172,10 +1172,10 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F23" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1203,10 +1203,10 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F24" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1234,10 +1234,10 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F25" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1265,10 +1265,10 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F26" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F27" t="n">
         <v>20261020</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,10 +1804,10 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F43" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,10 +1866,10 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F45" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49" t="n">
         <v>20261020</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F61" t="n">
         <v>20261020</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,10 +3296,10 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F91" t="n">
-        <v>20261011</v>
+        <v>20261021</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F94" t="n">
         <v>20261015</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Thu Oct 22 01:23:58 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>20261021</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
         <v>20261021</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
         <v>20261021</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F12" t="n">
         <v>20261021</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
         <v>20261021</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F22" t="n">
         <v>20261021</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
         <v>20261021</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F24" t="n">
         <v>20261021</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" t="n">
         <v>20261021</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F26" t="n">
         <v>20261021</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" t="n">
         <v>20261020</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F43" t="n">
         <v>20261021</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
         <v>20261021</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F49" t="n">
         <v>20261020</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F58" t="n">
         <v>20261013</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F59" t="n">
         <v>20261013</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" t="n">
         <v>20261013</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F61" t="n">
         <v>20261020</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F62" t="n">
         <v>20261013</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F63" t="n">
         <v>20261013</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F64" t="n">
         <v>20261013</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F91" t="n">
         <v>20261021</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,10 +3389,10 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F94" t="n">
-        <v>20261015</v>
+        <v>20261022</v>
       </c>
       <c r="G94" t="inlineStr"/>
       <c r="H94" t="inlineStr">
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Fri Oct 23 01:22:19 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
         <v>20261021</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
         <v>20261021</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
         <v>20261021</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F12" t="n">
         <v>20261021</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
         <v>20261021</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
         <v>20261014</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
         <v>20261014</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>20261014</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" t="n">
         <v>20261014</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F22" t="n">
         <v>20261021</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F23" t="n">
         <v>20261021</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F24" t="n">
         <v>20261021</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F25" t="n">
         <v>20261021</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F26" t="n">
         <v>20261021</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F27" t="n">
         <v>20261020</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" t="n">
         <v>20261014</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
         <v>20261014</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
         <v>20261014</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
         <v>20261014</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
         <v>20261014</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" t="n">
         <v>20261014</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="n">
         <v>20261014</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F35" t="n">
         <v>20261014</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F37" t="n">
         <v>20261014</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F38" t="n">
         <v>20261014</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F39" t="n">
         <v>20261014</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
         <v>20261014</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F43" t="n">
         <v>20261021</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F45" t="n">
         <v>20261021</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="n">
         <v>20261014</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F49" t="n">
         <v>20261020</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,10 +2273,10 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F58" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr">
@@ -2304,10 +2304,10 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F59" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2335,10 +2335,10 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F61" t="n">
         <v>20261020</v>
@@ -2397,10 +2397,10 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F62" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2428,10 +2428,10 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F63" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2459,10 +2459,10 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F64" t="n">
-        <v>20261013</v>
+        <v>20261023</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F65" t="n">
         <v>20261014</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F66" t="n">
         <v>20261014</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F67" t="n">
         <v>20261014</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" t="n">
         <v>20261014</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" t="n">
         <v>20261014</v>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F91" t="n">
         <v>20261021</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F94" t="n">
         <v>20261022</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sat Oct 24 01:27:58 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" t="n">
         <v>20261021</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F7" t="n">
         <v>20261021</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" t="n">
         <v>20261021</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>20261021</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" t="n">
         <v>20261015</v>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
         <v>20261021</v>
@@ -1017,10 +1017,10 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1048,10 +1048,10 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F19" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F20" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1110,10 +1110,10 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F21" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F22" t="n">
         <v>20261021</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
         <v>20261021</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F24" t="n">
         <v>20261021</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
         <v>20261021</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F26" t="n">
         <v>20261021</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F27" t="n">
         <v>20261020</v>
@@ -1331,10 +1331,10 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F28" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1362,10 +1362,10 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F29" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1393,10 +1393,10 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F30" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1424,10 +1424,10 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F31" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1455,10 +1455,10 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F32" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F33" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1517,10 +1517,10 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1552,10 +1552,10 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1614,10 +1614,10 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1645,10 +1645,10 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1676,10 +1676,10 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,10 +1773,10 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F42" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F43" t="n">
         <v>20261021</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F45" t="n">
         <v>20261021</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,10 +1932,10 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F47" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F49" t="n">
         <v>20261020</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F58" t="n">
         <v>20261023</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F59" t="n">
         <v>20261023</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F60" t="n">
         <v>20261023</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F61" t="n">
         <v>20261020</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F62" t="n">
         <v>20261023</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F63" t="n">
         <v>20261023</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F64" t="n">
         <v>20261023</v>
@@ -2490,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F65" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F66" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr">
@@ -2552,10 +2552,10 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr">
@@ -2583,10 +2583,10 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F68" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -2614,10 +2614,10 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F69" t="n">
-        <v>20261014</v>
+        <v>20261024</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -2645,7 +2645,7 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F70" t="n">
         <v>20261015</v>
@@ -2676,7 +2676,7 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F71" t="n">
         <v>20261015</v>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F72" t="n">
         <v>20261015</v>
@@ -2738,7 +2738,7 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="n">
         <v>20261015</v>
@@ -2769,7 +2769,7 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F74" t="n">
         <v>20261015</v>
@@ -2800,7 +2800,7 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F75" t="n">
         <v>20261015</v>
@@ -2831,7 +2831,7 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="n">
         <v>20261015</v>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F91" t="n">
         <v>20261021</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F94" t="n">
         <v>20261022</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,7 +3451,7 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F96" t="n">
         <v>20261015</v>
@@ -3482,7 +3482,7 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F97" t="n">
         <v>20261015</v>
@@ -3513,7 +3513,7 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F98" t="n">
         <v>20261015</v>
@@ -3544,7 +3544,7 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F99" t="n">
         <v>20261015</v>

</xml_diff>

<commit_message>
自动更新Excel文件 - Sun Oct 25 00:58:34 UTC 2026
</commit_message>
<xml_diff>
--- a/yxc_backup.xlsx
+++ b/yxc_backup.xlsx
@@ -493,7 +493,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n">
         <v>20261019</v>
@@ -528,7 +528,7 @@
         <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F3" t="n">
         <v>20261019</v>
@@ -563,7 +563,7 @@
         <v>14</v>
       </c>
       <c r="E4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n">
         <v>20261019</v>
@@ -598,7 +598,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
         <v>20261021</v>
@@ -633,7 +633,7 @@
         <v>14</v>
       </c>
       <c r="E6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n">
         <v>20261019</v>
@@ -664,7 +664,7 @@
         <v>10</v>
       </c>
       <c r="E7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>20261021</v>
@@ -695,7 +695,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" t="n">
         <v>20261019</v>
@@ -726,7 +726,7 @@
         <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F9" t="n">
         <v>20261021</v>
@@ -757,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F10" t="n">
         <v>20261019</v>
@@ -788,7 +788,7 @@
         <v>14</v>
       </c>
       <c r="E11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11" t="n">
         <v>20261019</v>
@@ -819,7 +819,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" t="n">
         <v>20261021</v>
@@ -850,7 +850,7 @@
         <v>14</v>
       </c>
       <c r="E13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F13" t="n">
         <v>20261019</v>
@@ -885,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
         <v>20261019</v>
@@ -920,7 +920,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F15" t="n">
         <v>20261019</v>
@@ -955,10 +955,10 @@
         <v>10</v>
       </c>
       <c r="E16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
         <v>10</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" t="n">
         <v>20261021</v>
@@ -1017,7 +1017,7 @@
         <v>10</v>
       </c>
       <c r="E18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18" t="n">
         <v>20261024</v>
@@ -1048,7 +1048,7 @@
         <v>10</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
         <v>20261024</v>
@@ -1079,7 +1079,7 @@
         <v>10</v>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F20" t="n">
         <v>20261024</v>
@@ -1110,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
         <v>20261024</v>
@@ -1141,7 +1141,7 @@
         <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
         <v>20261021</v>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
         <v>20261021</v>
@@ -1203,7 +1203,7 @@
         <v>10</v>
       </c>
       <c r="E24" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F24" t="n">
         <v>20261021</v>
@@ -1234,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" t="n">
         <v>20261021</v>
@@ -1265,7 +1265,7 @@
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
         <v>20261021</v>
@@ -1296,7 +1296,7 @@
         <v>7</v>
       </c>
       <c r="E27" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" t="n">
         <v>20261020</v>
@@ -1331,7 +1331,7 @@
         <v>10</v>
       </c>
       <c r="E28" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
         <v>20261024</v>
@@ -1362,7 +1362,7 @@
         <v>10</v>
       </c>
       <c r="E29" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
         <v>20261024</v>
@@ -1393,7 +1393,7 @@
         <v>10</v>
       </c>
       <c r="E30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F30" t="n">
         <v>20261024</v>
@@ -1424,7 +1424,7 @@
         <v>10</v>
       </c>
       <c r="E31" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F31" t="n">
         <v>20261024</v>
@@ -1455,7 +1455,7 @@
         <v>10</v>
       </c>
       <c r="E32" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F32" t="n">
         <v>20261024</v>
@@ -1486,7 +1486,7 @@
         <v>10</v>
       </c>
       <c r="E33" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" t="n">
         <v>20261024</v>
@@ -1517,7 +1517,7 @@
         <v>10</v>
       </c>
       <c r="E34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F34" t="n">
         <v>20261024</v>
@@ -1552,7 +1552,7 @@
         <v>10</v>
       </c>
       <c r="E35" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F35" t="n">
         <v>20261024</v>
@@ -1614,7 +1614,7 @@
         <v>10</v>
       </c>
       <c r="E37" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F37" t="n">
         <v>20261024</v>
@@ -1645,7 +1645,7 @@
         <v>10</v>
       </c>
       <c r="E38" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38" t="n">
         <v>20261024</v>
@@ -1676,7 +1676,7 @@
         <v>10</v>
       </c>
       <c r="E39" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" t="n">
         <v>20261024</v>
@@ -1711,7 +1711,7 @@
         <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F40" t="n">
         <v>20261019</v>
@@ -1742,7 +1742,7 @@
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
         <v>20261019</v>
@@ -1773,7 +1773,7 @@
         <v>10</v>
       </c>
       <c r="E42" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F42" t="n">
         <v>20261024</v>
@@ -1804,7 +1804,7 @@
         <v>10</v>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F43" t="n">
         <v>20261021</v>
@@ -1835,7 +1835,7 @@
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="n">
         <v>20261019</v>
@@ -1866,7 +1866,7 @@
         <v>10</v>
       </c>
       <c r="E45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F45" t="n">
         <v>20261021</v>
@@ -1897,7 +1897,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="n">
         <v>20261019</v>
@@ -1932,7 +1932,7 @@
         <v>10</v>
       </c>
       <c r="E47" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F47" t="n">
         <v>20261024</v>
@@ -1963,7 +1963,7 @@
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="n">
         <v>20261019</v>
@@ -1994,7 +1994,7 @@
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F49" t="n">
         <v>20261020</v>
@@ -2025,7 +2025,7 @@
         <v>10</v>
       </c>
       <c r="E50" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F50" t="n">
         <v>20261019</v>
@@ -2056,7 +2056,7 @@
         <v>10</v>
       </c>
       <c r="E51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F51" t="n">
         <v>20261019</v>
@@ -2087,7 +2087,7 @@
         <v>10</v>
       </c>
       <c r="E52" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
         <v>20261019</v>
@@ -2118,7 +2118,7 @@
         <v>10</v>
       </c>
       <c r="E53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F53" t="n">
         <v>20261019</v>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F54" t="n">
         <v>20261019</v>
@@ -2180,7 +2180,7 @@
         <v>10</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F55" t="n">
         <v>20261019</v>
@@ -2211,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F56" t="n">
         <v>20261019</v>
@@ -2242,7 +2242,7 @@
         <v>10</v>
       </c>
       <c r="E57" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F57" t="n">
         <v>20261019</v>
@@ -2273,7 +2273,7 @@
         <v>10</v>
       </c>
       <c r="E58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F58" t="n">
         <v>20261023</v>
@@ -2304,7 +2304,7 @@
         <v>10</v>
       </c>
       <c r="E59" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F59" t="n">
         <v>20261023</v>
@@ -2335,7 +2335,7 @@
         <v>10</v>
       </c>
       <c r="E60" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F60" t="n">
         <v>20261023</v>
@@ -2366,7 +2366,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F61" t="n">
         <v>20261020</v>
@@ -2397,7 +2397,7 @@
         <v>10</v>
       </c>
       <c r="E62" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F62" t="n">
         <v>20261023</v>
@@ -2428,7 +2428,7 @@
         <v>10</v>
       </c>
       <c r="E63" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F63" t="n">
         <v>20261023</v>
@@ -2459,7 +2459,7 @@
         <v>10</v>
       </c>
       <c r="E64" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F64" t="n">
         <v>20261023</v>
@@ -2490,7 +2490,7 @@
         <v>10</v>
       </c>
       <c r="E65" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F65" t="n">
         <v>20261024</v>
@@ -2521,7 +2521,7 @@
         <v>10</v>
       </c>
       <c r="E66" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F66" t="n">
         <v>20261024</v>
@@ -2552,7 +2552,7 @@
         <v>10</v>
       </c>
       <c r="E67" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F67" t="n">
         <v>20261024</v>
@@ -2583,7 +2583,7 @@
         <v>10</v>
       </c>
       <c r="E68" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F68" t="n">
         <v>20261024</v>
@@ -2614,7 +2614,7 @@
         <v>10</v>
       </c>
       <c r="E69" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F69" t="n">
         <v>20261024</v>
@@ -2645,10 +2645,10 @@
         <v>10</v>
       </c>
       <c r="E70" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F70" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2676,10 +2676,10 @@
         <v>10</v>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F71" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         <v>10</v>
       </c>
       <c r="E72" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F72" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2738,10 +2738,10 @@
         <v>10</v>
       </c>
       <c r="E73" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F73" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -2769,10 +2769,10 @@
         <v>10</v>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F74" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -2800,10 +2800,10 @@
         <v>10</v>
       </c>
       <c r="E75" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F75" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>10</v>
       </c>
       <c r="E76" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F76" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -2862,7 +2862,7 @@
         <v>10</v>
       </c>
       <c r="E77" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F77" t="n">
         <v>20261018</v>
@@ -2893,7 +2893,7 @@
         <v>10</v>
       </c>
       <c r="E78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F78" t="n">
         <v>20261018</v>
@@ -2924,7 +2924,7 @@
         <v>10</v>
       </c>
       <c r="E79" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F79" t="n">
         <v>20261018</v>
@@ -2955,7 +2955,7 @@
         <v>10</v>
       </c>
       <c r="E80" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F80" t="n">
         <v>20261018</v>
@@ -2986,7 +2986,7 @@
         <v>10</v>
       </c>
       <c r="E81" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F81" t="n">
         <v>20261018</v>
@@ -3017,7 +3017,7 @@
         <v>10</v>
       </c>
       <c r="E82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F82" t="n">
         <v>20261018</v>
@@ -3048,7 +3048,7 @@
         <v>10</v>
       </c>
       <c r="E83" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F83" t="n">
         <v>20261018</v>
@@ -3079,7 +3079,7 @@
         <v>10</v>
       </c>
       <c r="E84" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F84" t="n">
         <v>20261018</v>
@@ -3110,7 +3110,7 @@
         <v>10</v>
       </c>
       <c r="E85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F85" t="n">
         <v>20261018</v>
@@ -3141,7 +3141,7 @@
         <v>10</v>
       </c>
       <c r="E86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F86" t="n">
         <v>20261018</v>
@@ -3172,7 +3172,7 @@
         <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="n">
         <v>20261019</v>
@@ -3203,7 +3203,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F88" t="n">
         <v>20261019</v>
@@ -3234,7 +3234,7 @@
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
         <v>20261019</v>
@@ -3265,7 +3265,7 @@
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F90" t="n">
         <v>20261019</v>
@@ -3296,7 +3296,7 @@
         <v>10</v>
       </c>
       <c r="E91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F91" t="n">
         <v>20261021</v>
@@ -3327,7 +3327,7 @@
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F92" t="n">
         <v>20261019</v>
@@ -3358,7 +3358,7 @@
         <v>10</v>
       </c>
       <c r="E93" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F93" t="n">
         <v>20261018</v>
@@ -3389,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F94" t="n">
         <v>20261022</v>
@@ -3420,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F95" t="n">
         <v>20261017</v>
@@ -3451,10 +3451,10 @@
         <v>10</v>
       </c>
       <c r="E96" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F96" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G96" t="inlineStr"/>
       <c r="H96" t="inlineStr">
@@ -3482,10 +3482,10 @@
         <v>10</v>
       </c>
       <c r="E97" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F97" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>10</v>
       </c>
       <c r="E98" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F98" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -3544,10 +3544,10 @@
         <v>10</v>
       </c>
       <c r="E99" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F99" t="n">
-        <v>20261015</v>
+        <v>20261025</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>

</xml_diff>